<commit_message>
Added water quality variable
</commit_message>
<xml_diff>
--- a/baza_balkany.xlsx
+++ b/baza_balkany.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H283"/>
+  <dimension ref="A1:I283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>Poziom_Cen_NUTS0</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Wody_Doskonała_Jakość_NUTS0</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -497,6 +502,9 @@
       <c r="H2" t="n">
         <v>49.4</v>
       </c>
+      <c r="I2" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -525,6 +533,9 @@
       <c r="H3" t="n">
         <v>49.4</v>
       </c>
+      <c r="I3" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,6 +564,9 @@
       <c r="H4" t="n">
         <v>49.4</v>
       </c>
+      <c r="I4" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -581,6 +595,9 @@
       <c r="H5" t="n">
         <v>47.6</v>
       </c>
+      <c r="I5" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -609,6 +626,9 @@
       <c r="H6" t="n">
         <v>47.6</v>
       </c>
+      <c r="I6" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -639,6 +659,9 @@
       <c r="H7" t="n">
         <v>47.6</v>
       </c>
+      <c r="I7" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -669,6 +692,9 @@
       <c r="H8" t="n">
         <v>47.6</v>
       </c>
+      <c r="I8" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -699,6 +725,9 @@
       <c r="H9" t="n">
         <v>47.6</v>
       </c>
+      <c r="I9" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -727,6 +756,9 @@
       <c r="H10" t="n">
         <v>47.6</v>
       </c>
+      <c r="I10" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -757,6 +789,9 @@
       <c r="H11" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I11" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -787,6 +822,9 @@
       <c r="H12" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I12" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -817,6 +855,9 @@
       <c r="H13" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I13" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -847,6 +888,9 @@
       <c r="H14" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I14" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -877,6 +921,9 @@
       <c r="H15" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I15" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -907,6 +954,9 @@
       <c r="H16" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I16" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -937,6 +987,9 @@
       <c r="H17" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I17" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -967,6 +1020,9 @@
       <c r="H18" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I18" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -997,6 +1053,9 @@
       <c r="H19" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I19" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1027,6 +1086,9 @@
       <c r="H20" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I20" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1057,6 +1119,9 @@
       <c r="H21" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I21" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1087,6 +1152,9 @@
       <c r="H22" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I22" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1117,6 +1185,9 @@
       <c r="H23" t="n">
         <v>84.09999999999999</v>
       </c>
+      <c r="I23" t="n">
+        <v>1595</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1145,6 +1216,9 @@
       <c r="H24" t="n">
         <v>66.3</v>
       </c>
+      <c r="I24" t="n">
+        <v>981</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1175,6 +1249,9 @@
       <c r="H25" t="n">
         <v>66.3</v>
       </c>
+      <c r="I25" t="n">
+        <v>981</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1203,6 +1280,9 @@
       <c r="H26" t="n">
         <v>66.3</v>
       </c>
+      <c r="I26" t="n">
+        <v>981</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1231,6 +1311,9 @@
       <c r="H27" t="n">
         <v>66.3</v>
       </c>
+      <c r="I27" t="n">
+        <v>981</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1261,6 +1344,9 @@
       <c r="H28" t="n">
         <v>66.3</v>
       </c>
+      <c r="I28" t="n">
+        <v>981</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1291,6 +1377,7 @@
       <c r="H29" t="n">
         <v>44.9</v>
       </c>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1321,6 +1408,9 @@
       <c r="H30" t="n">
         <v>50.4</v>
       </c>
+      <c r="I30" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1351,6 +1441,9 @@
       <c r="H31" t="n">
         <v>50.4</v>
       </c>
+      <c r="I31" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1381,6 +1474,9 @@
       <c r="H32" t="n">
         <v>50.4</v>
       </c>
+      <c r="I32" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1409,6 +1505,9 @@
       <c r="H33" t="n">
         <v>50.4</v>
       </c>
+      <c r="I33" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1437,6 +1536,9 @@
       <c r="H34" t="n">
         <v>50.4</v>
       </c>
+      <c r="I34" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1467,6 +1569,9 @@
       <c r="H35" t="n">
         <v>50.4</v>
       </c>
+      <c r="I35" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1497,6 +1602,9 @@
       <c r="H36" t="n">
         <v>50.4</v>
       </c>
+      <c r="I36" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1527,6 +1635,9 @@
       <c r="H37" t="n">
         <v>50.4</v>
       </c>
+      <c r="I37" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1555,6 +1666,9 @@
       <c r="H38" t="n">
         <v>51.7</v>
       </c>
+      <c r="I38" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1583,6 +1697,9 @@
       <c r="H39" t="n">
         <v>51.7</v>
       </c>
+      <c r="I39" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1611,6 +1728,9 @@
       <c r="H40" t="n">
         <v>51.7</v>
       </c>
+      <c r="I40" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1639,6 +1759,9 @@
       <c r="H41" t="n">
         <v>49.4</v>
       </c>
+      <c r="I41" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1667,6 +1790,9 @@
       <c r="H42" t="n">
         <v>49.4</v>
       </c>
+      <c r="I42" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1697,6 +1823,9 @@
       <c r="H43" t="n">
         <v>49.4</v>
       </c>
+      <c r="I43" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1727,6 +1856,9 @@
       <c r="H44" t="n">
         <v>49.4</v>
       </c>
+      <c r="I44" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1757,6 +1889,9 @@
       <c r="H45" t="n">
         <v>49.4</v>
       </c>
+      <c r="I45" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1785,6 +1920,9 @@
       <c r="H46" t="n">
         <v>49.4</v>
       </c>
+      <c r="I46" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1815,6 +1953,9 @@
       <c r="H47" t="n">
         <v>84.8</v>
       </c>
+      <c r="I47" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1845,6 +1986,9 @@
       <c r="H48" t="n">
         <v>84.8</v>
       </c>
+      <c r="I48" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1875,6 +2019,9 @@
       <c r="H49" t="n">
         <v>84.8</v>
       </c>
+      <c r="I49" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1905,6 +2052,9 @@
       <c r="H50" t="n">
         <v>84.8</v>
       </c>
+      <c r="I50" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1935,6 +2085,9 @@
       <c r="H51" t="n">
         <v>84.8</v>
       </c>
+      <c r="I51" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1965,6 +2118,9 @@
       <c r="H52" t="n">
         <v>84.8</v>
       </c>
+      <c r="I52" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1995,6 +2151,9 @@
       <c r="H53" t="n">
         <v>84.8</v>
       </c>
+      <c r="I53" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2025,6 +2184,9 @@
       <c r="H54" t="n">
         <v>84.8</v>
       </c>
+      <c r="I54" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2055,6 +2217,9 @@
       <c r="H55" t="n">
         <v>84.8</v>
       </c>
+      <c r="I55" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2085,6 +2250,9 @@
       <c r="H56" t="n">
         <v>84.8</v>
       </c>
+      <c r="I56" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2115,6 +2283,9 @@
       <c r="H57" t="n">
         <v>84.8</v>
       </c>
+      <c r="I57" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2145,6 +2316,9 @@
       <c r="H58" t="n">
         <v>84.8</v>
       </c>
+      <c r="I58" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2175,6 +2349,9 @@
       <c r="H59" t="n">
         <v>84.8</v>
       </c>
+      <c r="I59" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2203,6 +2380,9 @@
       <c r="H60" t="n">
         <v>67</v>
       </c>
+      <c r="I60" t="n">
+        <v>953</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2233,6 +2413,9 @@
       <c r="H61" t="n">
         <v>67</v>
       </c>
+      <c r="I61" t="n">
+        <v>953</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2261,6 +2444,9 @@
       <c r="H62" t="n">
         <v>67</v>
       </c>
+      <c r="I62" t="n">
+        <v>953</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2289,6 +2475,9 @@
       <c r="H63" t="n">
         <v>67</v>
       </c>
+      <c r="I63" t="n">
+        <v>953</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2319,6 +2508,9 @@
       <c r="H64" t="n">
         <v>67</v>
       </c>
+      <c r="I64" t="n">
+        <v>953</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2349,6 +2541,7 @@
       <c r="H65" t="n">
         <v>45.3</v>
       </c>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2379,6 +2572,9 @@
       <c r="H66" t="n">
         <v>50.4</v>
       </c>
+      <c r="I66" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2409,6 +2605,9 @@
       <c r="H67" t="n">
         <v>50.4</v>
       </c>
+      <c r="I67" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2439,6 +2638,9 @@
       <c r="H68" t="n">
         <v>50.4</v>
       </c>
+      <c r="I68" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2469,6 +2671,9 @@
       <c r="H69" t="n">
         <v>50.4</v>
       </c>
+      <c r="I69" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2497,6 +2702,9 @@
       <c r="H70" t="n">
         <v>50.4</v>
       </c>
+      <c r="I70" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2527,6 +2735,9 @@
       <c r="H71" t="n">
         <v>50.4</v>
       </c>
+      <c r="I71" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2557,6 +2768,9 @@
       <c r="H72" t="n">
         <v>50.4</v>
       </c>
+      <c r="I72" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2587,6 +2801,9 @@
       <c r="H73" t="n">
         <v>50.4</v>
       </c>
+      <c r="I73" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2615,6 +2832,9 @@
       <c r="H74" t="n">
         <v>86.40000000000001</v>
       </c>
+      <c r="I74" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2645,6 +2865,9 @@
       <c r="H75" t="n">
         <v>86.40000000000001</v>
       </c>
+      <c r="I75" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2673,6 +2896,9 @@
       <c r="H76" t="n">
         <v>52.5</v>
       </c>
+      <c r="I76" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2701,6 +2927,9 @@
       <c r="H77" t="n">
         <v>52.5</v>
       </c>
+      <c r="I77" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2729,6 +2958,9 @@
       <c r="H78" t="n">
         <v>52.5</v>
       </c>
+      <c r="I78" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2757,6 +2989,9 @@
       <c r="H79" t="n">
         <v>51.3</v>
       </c>
+      <c r="I79" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2785,6 +3020,9 @@
       <c r="H80" t="n">
         <v>51.3</v>
       </c>
+      <c r="I80" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2815,6 +3053,9 @@
       <c r="H81" t="n">
         <v>51.3</v>
       </c>
+      <c r="I81" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2845,6 +3086,9 @@
       <c r="H82" t="n">
         <v>51.3</v>
       </c>
+      <c r="I82" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2875,6 +3119,9 @@
       <c r="H83" t="n">
         <v>51.3</v>
       </c>
+      <c r="I83" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2903,6 +3150,9 @@
       <c r="H84" t="n">
         <v>51.3</v>
       </c>
+      <c r="I84" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2933,6 +3183,9 @@
       <c r="H85" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I85" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2963,6 +3216,9 @@
       <c r="H86" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I86" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2993,6 +3249,9 @@
       <c r="H87" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I87" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3023,6 +3282,9 @@
       <c r="H88" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I88" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3053,6 +3315,9 @@
       <c r="H89" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I89" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3083,6 +3348,9 @@
       <c r="H90" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I90" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3113,6 +3381,9 @@
       <c r="H91" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I91" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3143,6 +3414,9 @@
       <c r="H92" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I92" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3173,6 +3447,9 @@
       <c r="H93" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I93" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3203,6 +3480,9 @@
       <c r="H94" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I94" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3233,6 +3513,9 @@
       <c r="H95" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I95" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3263,6 +3546,9 @@
       <c r="H96" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I96" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3293,6 +3579,9 @@
       <c r="H97" t="n">
         <v>85.09999999999999</v>
       </c>
+      <c r="I97" t="n">
+        <v>1631</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3321,6 +3610,9 @@
       <c r="H98" t="n">
         <v>66.09999999999999</v>
       </c>
+      <c r="I98" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3351,6 +3643,9 @@
       <c r="H99" t="n">
         <v>66.09999999999999</v>
       </c>
+      <c r="I99" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3379,6 +3674,9 @@
       <c r="H100" t="n">
         <v>66.09999999999999</v>
       </c>
+      <c r="I100" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3409,6 +3707,9 @@
       <c r="H101" t="n">
         <v>66.09999999999999</v>
       </c>
+      <c r="I101" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3439,6 +3740,7 @@
       <c r="H102" t="n">
         <v>46.3</v>
       </c>
+      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3469,6 +3771,9 @@
       <c r="H103" t="n">
         <v>49.4</v>
       </c>
+      <c r="I103" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3499,6 +3804,9 @@
       <c r="H104" t="n">
         <v>49.4</v>
       </c>
+      <c r="I104" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3529,6 +3837,9 @@
       <c r="H105" t="n">
         <v>49.4</v>
       </c>
+      <c r="I105" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3557,6 +3868,9 @@
       <c r="H106" t="n">
         <v>49.4</v>
       </c>
+      <c r="I106" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3585,6 +3899,9 @@
       <c r="H107" t="n">
         <v>49.4</v>
       </c>
+      <c r="I107" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3615,6 +3932,9 @@
       <c r="H108" t="n">
         <v>49.4</v>
       </c>
+      <c r="I108" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3645,6 +3965,9 @@
       <c r="H109" t="n">
         <v>49.4</v>
       </c>
+      <c r="I109" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3674,6 +3997,9 @@
       </c>
       <c r="H110" t="n">
         <v>49.4</v>
+      </c>
+      <c r="I110" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="111">
@@ -3703,6 +4029,7 @@
       <c r="H111" t="n">
         <v>52.1</v>
       </c>
+      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3729,6 +4056,7 @@
       <c r="H112" t="n">
         <v>52.1</v>
       </c>
+      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3755,6 +4083,7 @@
       <c r="H113" t="n">
         <v>52.1</v>
       </c>
+      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3783,6 +4112,7 @@
       <c r="H114" t="n">
         <v>52.1</v>
       </c>
+      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3809,6 +4139,9 @@
       <c r="H115" t="n">
         <v>86.3</v>
       </c>
+      <c r="I115" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3837,6 +4170,9 @@
       <c r="H116" t="n">
         <v>86.3</v>
       </c>
+      <c r="I116" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3865,6 +4201,9 @@
       <c r="H117" t="n">
         <v>54.2</v>
       </c>
+      <c r="I117" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3893,6 +4232,9 @@
       <c r="H118" t="n">
         <v>54.2</v>
       </c>
+      <c r="I118" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3921,6 +4263,9 @@
       <c r="H119" t="n">
         <v>54.2</v>
       </c>
+      <c r="I119" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3949,6 +4294,9 @@
       <c r="H120" t="n">
         <v>51.6</v>
       </c>
+      <c r="I120" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3977,6 +4325,9 @@
       <c r="H121" t="n">
         <v>51.6</v>
       </c>
+      <c r="I121" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4007,6 +4358,9 @@
       <c r="H122" t="n">
         <v>51.6</v>
       </c>
+      <c r="I122" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4037,6 +4391,9 @@
       <c r="H123" t="n">
         <v>51.6</v>
       </c>
+      <c r="I123" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4067,6 +4424,9 @@
       <c r="H124" t="n">
         <v>51.6</v>
       </c>
+      <c r="I124" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4095,6 +4455,9 @@
       <c r="H125" t="n">
         <v>51.6</v>
       </c>
+      <c r="I125" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4125,6 +4488,9 @@
       <c r="H126" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I126" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4155,6 +4521,9 @@
       <c r="H127" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I127" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4185,6 +4554,9 @@
       <c r="H128" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I128" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4215,6 +4587,9 @@
       <c r="H129" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I129" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4245,6 +4620,9 @@
       <c r="H130" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I130" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4275,6 +4653,9 @@
       <c r="H131" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I131" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4305,6 +4686,9 @@
       <c r="H132" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I132" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4335,6 +4719,9 @@
       <c r="H133" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I133" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4365,6 +4752,9 @@
       <c r="H134" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I134" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4395,6 +4785,9 @@
       <c r="H135" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I135" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4425,6 +4818,9 @@
       <c r="H136" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I136" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4455,6 +4851,9 @@
       <c r="H137" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I137" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4485,6 +4884,9 @@
       <c r="H138" t="n">
         <v>83.90000000000001</v>
       </c>
+      <c r="I138" t="n">
+        <v>1680</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4513,6 +4915,9 @@
       <c r="H139" t="n">
         <v>65.2</v>
       </c>
+      <c r="I139" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4543,6 +4948,9 @@
       <c r="H140" t="n">
         <v>65.2</v>
       </c>
+      <c r="I140" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4571,6 +4979,9 @@
       <c r="H141" t="n">
         <v>65.2</v>
       </c>
+      <c r="I141" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4601,6 +5012,9 @@
       <c r="H142" t="n">
         <v>65.2</v>
       </c>
+      <c r="I142" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4631,6 +5045,7 @@
       <c r="H143" t="n">
         <v>44.6</v>
       </c>
+      <c r="I143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4661,6 +5076,9 @@
       <c r="H144" t="n">
         <v>49.7</v>
       </c>
+      <c r="I144" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4691,6 +5109,9 @@
       <c r="H145" t="n">
         <v>49.7</v>
       </c>
+      <c r="I145" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4721,6 +5142,9 @@
       <c r="H146" t="n">
         <v>49.7</v>
       </c>
+      <c r="I146" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4751,6 +5175,9 @@
       <c r="H147" t="n">
         <v>49.7</v>
       </c>
+      <c r="I147" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4779,6 +5206,9 @@
       <c r="H148" t="n">
         <v>49.7</v>
       </c>
+      <c r="I148" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4809,6 +5239,9 @@
       <c r="H149" t="n">
         <v>49.7</v>
       </c>
+      <c r="I149" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4839,6 +5272,9 @@
       <c r="H150" t="n">
         <v>49.7</v>
       </c>
+      <c r="I150" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4869,6 +5305,9 @@
       <c r="H151" t="n">
         <v>49.7</v>
       </c>
+      <c r="I151" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4899,6 +5338,7 @@
       <c r="H152" t="n">
         <v>54</v>
       </c>
+      <c r="I152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4927,6 +5367,7 @@
       <c r="H153" t="n">
         <v>54</v>
       </c>
+      <c r="I153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4955,6 +5396,7 @@
       <c r="H154" t="n">
         <v>54</v>
       </c>
+      <c r="I154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4985,6 +5427,7 @@
       <c r="H155" t="n">
         <v>54</v>
       </c>
+      <c r="I155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5013,6 +5456,9 @@
       <c r="H156" t="n">
         <v>87.2</v>
       </c>
+      <c r="I156" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5043,6 +5489,9 @@
       <c r="H157" t="n">
         <v>87.2</v>
       </c>
+      <c r="I157" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5071,6 +5520,9 @@
       <c r="H158" t="n">
         <v>54.6</v>
       </c>
+      <c r="I158" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5099,6 +5551,9 @@
       <c r="H159" t="n">
         <v>54.6</v>
       </c>
+      <c r="I159" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5127,6 +5582,9 @@
       <c r="H160" t="n">
         <v>54.6</v>
       </c>
+      <c r="I160" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5155,6 +5613,9 @@
       <c r="H161" t="n">
         <v>54.3</v>
       </c>
+      <c r="I161" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5183,6 +5644,9 @@
       <c r="H162" t="n">
         <v>54.3</v>
       </c>
+      <c r="I162" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5213,6 +5677,9 @@
       <c r="H163" t="n">
         <v>54.3</v>
       </c>
+      <c r="I163" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5243,6 +5710,9 @@
       <c r="H164" t="n">
         <v>54.3</v>
       </c>
+      <c r="I164" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5273,6 +5743,9 @@
       <c r="H165" t="n">
         <v>54.3</v>
       </c>
+      <c r="I165" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5301,6 +5774,9 @@
       <c r="H166" t="n">
         <v>54.3</v>
       </c>
+      <c r="I166" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5331,6 +5807,9 @@
       <c r="H167" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I167" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5361,6 +5840,9 @@
       <c r="H168" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I168" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5391,6 +5873,9 @@
       <c r="H169" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I169" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5421,6 +5906,9 @@
       <c r="H170" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I170" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5451,6 +5939,9 @@
       <c r="H171" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I171" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5481,6 +5972,9 @@
       <c r="H172" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I172" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5511,6 +6005,9 @@
       <c r="H173" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I173" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5541,6 +6038,9 @@
       <c r="H174" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I174" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5571,6 +6071,9 @@
       <c r="H175" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I175" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5601,6 +6104,9 @@
       <c r="H176" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I176" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5631,6 +6137,9 @@
       <c r="H177" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I177" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5661,6 +6170,9 @@
       <c r="H178" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I178" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5691,6 +6203,9 @@
       <c r="H179" t="n">
         <v>84.40000000000001</v>
       </c>
+      <c r="I179" t="n">
+        <v>1679</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5719,6 +6234,9 @@
       <c r="H180" t="n">
         <v>68.5</v>
       </c>
+      <c r="I180" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5749,6 +6267,9 @@
       <c r="H181" t="n">
         <v>68.5</v>
       </c>
+      <c r="I181" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5777,6 +6298,9 @@
       <c r="H182" t="n">
         <v>68.5</v>
       </c>
+      <c r="I182" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5807,6 +6331,9 @@
       <c r="H183" t="n">
         <v>68.5</v>
       </c>
+      <c r="I183" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5837,6 +6364,7 @@
       <c r="H184" t="n">
         <v>55.8</v>
       </c>
+      <c r="I184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5867,6 +6395,7 @@
       <c r="H185" t="n">
         <v>47.2</v>
       </c>
+      <c r="I185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -5897,6 +6426,9 @@
       <c r="H186" t="n">
         <v>53.2</v>
       </c>
+      <c r="I186" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5927,6 +6459,9 @@
       <c r="H187" t="n">
         <v>53.2</v>
       </c>
+      <c r="I187" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5957,6 +6492,9 @@
       <c r="H188" t="n">
         <v>53.2</v>
       </c>
+      <c r="I188" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5985,6 +6523,9 @@
       <c r="H189" t="n">
         <v>53.2</v>
       </c>
+      <c r="I189" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6013,6 +6554,9 @@
       <c r="H190" t="n">
         <v>53.2</v>
       </c>
+      <c r="I190" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6043,6 +6587,9 @@
       <c r="H191" t="n">
         <v>53.2</v>
       </c>
+      <c r="I191" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6073,6 +6620,9 @@
       <c r="H192" t="n">
         <v>53.2</v>
       </c>
+      <c r="I192" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6103,6 +6653,9 @@
       <c r="H193" t="n">
         <v>53.2</v>
       </c>
+      <c r="I193" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6133,6 +6686,7 @@
       <c r="H194" t="n">
         <v>57</v>
       </c>
+      <c r="I194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6161,6 +6715,7 @@
       <c r="H195" t="n">
         <v>57</v>
       </c>
+      <c r="I195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6189,6 +6744,7 @@
       <c r="H196" t="n">
         <v>57</v>
       </c>
+      <c r="I196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6219,6 +6775,7 @@
       <c r="H197" t="n">
         <v>57</v>
       </c>
+      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6247,6 +6804,9 @@
       <c r="H198" t="n">
         <v>87.8</v>
       </c>
+      <c r="I198" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6277,6 +6837,9 @@
       <c r="H199" t="n">
         <v>87.8</v>
       </c>
+      <c r="I199" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6304,6 +6867,9 @@
       </c>
       <c r="H200" t="n">
         <v>58.2</v>
+      </c>
+      <c r="I200" t="n">
+        <v>113</v>
       </c>
     </row>
     <row r="201">
@@ -6331,6 +6897,9 @@
       <c r="H201" t="n">
         <v>58.2</v>
       </c>
+      <c r="I201" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6358,6 +6927,9 @@
       </c>
       <c r="H202" t="n">
         <v>58.2</v>
+      </c>
+      <c r="I202" t="n">
+        <v>113</v>
       </c>
     </row>
     <row r="203">
@@ -6385,6 +6957,9 @@
       <c r="H203" t="n">
         <v>55.8</v>
       </c>
+      <c r="I203" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -6411,6 +6986,9 @@
       <c r="H204" t="n">
         <v>55.8</v>
       </c>
+      <c r="I204" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6441,6 +7019,9 @@
       <c r="H205" t="n">
         <v>55.8</v>
       </c>
+      <c r="I205" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -6471,6 +7052,9 @@
       <c r="H206" t="n">
         <v>55.8</v>
       </c>
+      <c r="I206" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6501,6 +7085,9 @@
       <c r="H207" t="n">
         <v>55.8</v>
       </c>
+      <c r="I207" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6529,6 +7116,9 @@
       <c r="H208" t="n">
         <v>55.8</v>
       </c>
+      <c r="I208" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6559,6 +7149,9 @@
       <c r="H209" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I209" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6589,6 +7182,9 @@
       <c r="H210" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I210" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6619,6 +7215,9 @@
       <c r="H211" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I211" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6649,6 +7248,9 @@
       <c r="H212" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I212" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6679,6 +7281,9 @@
       <c r="H213" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I213" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6709,6 +7314,9 @@
       <c r="H214" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I214" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6739,6 +7347,9 @@
       <c r="H215" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I215" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6769,6 +7380,9 @@
       <c r="H216" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I216" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6799,6 +7413,9 @@
       <c r="H217" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I217" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6829,6 +7446,9 @@
       <c r="H218" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I218" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6859,6 +7479,9 @@
       <c r="H219" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I219" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6889,6 +7512,9 @@
       <c r="H220" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I220" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6919,6 +7545,9 @@
       <c r="H221" t="n">
         <v>82.90000000000001</v>
       </c>
+      <c r="I221" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6947,6 +7576,9 @@
       <c r="H222" t="n">
         <v>71.2</v>
       </c>
+      <c r="I222" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -6977,6 +7609,9 @@
       <c r="H223" t="n">
         <v>71.2</v>
       </c>
+      <c r="I223" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -7005,6 +7640,9 @@
       <c r="H224" t="n">
         <v>71.2</v>
       </c>
+      <c r="I224" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -7035,6 +7673,9 @@
       <c r="H225" t="n">
         <v>71.2</v>
       </c>
+      <c r="I225" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -7065,6 +7706,7 @@
       <c r="H226" t="n">
         <v>56.8</v>
       </c>
+      <c r="I226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7095,6 +7737,7 @@
       <c r="H227" t="n">
         <v>48.7</v>
       </c>
+      <c r="I227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7125,6 +7768,9 @@
       <c r="H228" t="n">
         <v>54.7</v>
       </c>
+      <c r="I228" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7155,6 +7801,9 @@
       <c r="H229" t="n">
         <v>54.7</v>
       </c>
+      <c r="I229" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7185,6 +7834,9 @@
       <c r="H230" t="n">
         <v>54.7</v>
       </c>
+      <c r="I230" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7213,6 +7865,9 @@
       <c r="H231" t="n">
         <v>54.7</v>
       </c>
+      <c r="I231" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7241,6 +7896,9 @@
       <c r="H232" t="n">
         <v>54.7</v>
       </c>
+      <c r="I232" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7271,6 +7929,9 @@
       <c r="H233" t="n">
         <v>54.7</v>
       </c>
+      <c r="I233" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7301,6 +7962,9 @@
       <c r="H234" t="n">
         <v>54.7</v>
       </c>
+      <c r="I234" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -7331,6 +7995,9 @@
       <c r="H235" t="n">
         <v>54.7</v>
       </c>
+      <c r="I235" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -7361,6 +8028,7 @@
       <c r="H236" t="n">
         <v>59.3</v>
       </c>
+      <c r="I236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -7389,6 +8057,7 @@
       <c r="H237" t="n">
         <v>59.3</v>
       </c>
+      <c r="I237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -7417,6 +8086,7 @@
       <c r="H238" t="n">
         <v>59.3</v>
       </c>
+      <c r="I238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -7447,6 +8117,7 @@
       <c r="H239" t="n">
         <v>59.3</v>
       </c>
+      <c r="I239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -7475,6 +8146,9 @@
       <c r="H240" t="n">
         <v>89.90000000000001</v>
       </c>
+      <c r="I240" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -7505,6 +8179,9 @@
       <c r="H241" t="n">
         <v>89.90000000000001</v>
       </c>
+      <c r="I241" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -7533,6 +8210,9 @@
       <c r="H242" t="n">
         <v>62.9</v>
       </c>
+      <c r="I242" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -7561,6 +8241,9 @@
       <c r="H243" t="n">
         <v>62.9</v>
       </c>
+      <c r="I243" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -7589,6 +8272,9 @@
       <c r="H244" t="n">
         <v>62.9</v>
       </c>
+      <c r="I244" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -7617,6 +8303,9 @@
       <c r="H245" t="n">
         <v>56.9</v>
       </c>
+      <c r="I245" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -7645,6 +8334,9 @@
       <c r="H246" t="n">
         <v>56.9</v>
       </c>
+      <c r="I246" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -7675,6 +8367,9 @@
       <c r="H247" t="n">
         <v>56.9</v>
       </c>
+      <c r="I247" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -7705,6 +8400,9 @@
       <c r="H248" t="n">
         <v>56.9</v>
       </c>
+      <c r="I248" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -7735,6 +8433,9 @@
       <c r="H249" t="n">
         <v>56.9</v>
       </c>
+      <c r="I249" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -7763,6 +8464,9 @@
       <c r="H250" t="n">
         <v>56.9</v>
       </c>
+      <c r="I250" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -7793,6 +8497,9 @@
       <c r="H251" t="n">
         <v>83</v>
       </c>
+      <c r="I251" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -7823,6 +8530,9 @@
       <c r="H252" t="n">
         <v>83</v>
       </c>
+      <c r="I252" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -7853,6 +8563,9 @@
       <c r="H253" t="n">
         <v>83</v>
       </c>
+      <c r="I253" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -7883,6 +8596,9 @@
       <c r="H254" t="n">
         <v>83</v>
       </c>
+      <c r="I254" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -7913,6 +8629,9 @@
       <c r="H255" t="n">
         <v>83</v>
       </c>
+      <c r="I255" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -7943,6 +8662,9 @@
       <c r="H256" t="n">
         <v>83</v>
       </c>
+      <c r="I256" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -7973,6 +8695,9 @@
       <c r="H257" t="n">
         <v>83</v>
       </c>
+      <c r="I257" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -8003,6 +8728,9 @@
       <c r="H258" t="n">
         <v>83</v>
       </c>
+      <c r="I258" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -8033,6 +8761,9 @@
       <c r="H259" t="n">
         <v>83</v>
       </c>
+      <c r="I259" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -8063,6 +8794,9 @@
       <c r="H260" t="n">
         <v>83</v>
       </c>
+      <c r="I260" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -8093,6 +8827,9 @@
       <c r="H261" t="n">
         <v>83</v>
       </c>
+      <c r="I261" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -8123,6 +8860,9 @@
       <c r="H262" t="n">
         <v>83</v>
       </c>
+      <c r="I262" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -8153,6 +8893,9 @@
       <c r="H263" t="n">
         <v>83</v>
       </c>
+      <c r="I263" t="n">
+        <v>1728</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -8181,6 +8924,9 @@
       <c r="H264" t="n">
         <v>73.3</v>
       </c>
+      <c r="I264" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -8211,6 +8957,9 @@
       <c r="H265" t="n">
         <v>73.3</v>
       </c>
+      <c r="I265" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -8239,6 +8988,9 @@
       <c r="H266" t="n">
         <v>73.3</v>
       </c>
+      <c r="I266" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -8269,6 +9021,9 @@
       <c r="H267" t="n">
         <v>73.3</v>
       </c>
+      <c r="I267" t="n">
+        <v>894</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -8299,6 +9054,7 @@
       <c r="H268" t="n">
         <v>57.9</v>
       </c>
+      <c r="I268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -8329,6 +9085,7 @@
       <c r="H269" t="n">
         <v>49.6</v>
       </c>
+      <c r="I269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -8359,6 +9116,9 @@
       <c r="H270" t="n">
         <v>57.4</v>
       </c>
+      <c r="I270" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -8389,6 +9149,9 @@
       <c r="H271" t="n">
         <v>57.4</v>
       </c>
+      <c r="I271" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -8419,6 +9182,9 @@
       <c r="H272" t="n">
         <v>57.4</v>
       </c>
+      <c r="I272" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -8447,6 +9213,9 @@
       <c r="H273" t="n">
         <v>57.4</v>
       </c>
+      <c r="I273" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -8475,6 +9244,9 @@
       <c r="H274" t="n">
         <v>57.4</v>
       </c>
+      <c r="I274" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -8505,6 +9277,9 @@
       <c r="H275" t="n">
         <v>57.4</v>
       </c>
+      <c r="I275" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -8535,6 +9310,9 @@
       <c r="H276" t="n">
         <v>57.4</v>
       </c>
+      <c r="I276" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -8565,6 +9343,9 @@
       <c r="H277" t="n">
         <v>57.4</v>
       </c>
+      <c r="I277" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -8595,6 +9376,7 @@
       <c r="H278" t="n">
         <v>61.4</v>
       </c>
+      <c r="I278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -8623,6 +9405,7 @@
       <c r="H279" t="n">
         <v>61.4</v>
       </c>
+      <c r="I279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -8651,6 +9434,7 @@
       <c r="H280" t="n">
         <v>61.4</v>
       </c>
+      <c r="I280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -8681,6 +9465,7 @@
       <c r="H281" t="n">
         <v>61.4</v>
       </c>
+      <c r="I281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -8709,6 +9494,9 @@
       <c r="H282" t="n">
         <v>91</v>
       </c>
+      <c r="I282" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -8738,6 +9526,9 @@
       </c>
       <c r="H283" t="n">
         <v>91</v>
+      </c>
+      <c r="I283" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>